<commit_message>
feat(governance): update Meeting 2 records, add workspace boundary audit tool and team git skills
</commit_message>
<xml_diff>
--- a/Meeting/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/Meeting/PI_GUARD_PROCESS_REPORT.xlsx
@@ -544,7 +544,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -552,21 +552,21 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
-    <col width="35" customWidth="1" min="11" max="11"/>
-    <col width="35" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
-    <col width="35" customWidth="1" min="14" max="14"/>
-    <col width="35" customWidth="1" min="15" max="15"/>
-    <col width="35" customWidth="1" min="16" max="16"/>
-    <col width="35" customWidth="1" min="17" max="17"/>
-    <col width="35" customWidth="1" min="18" max="18"/>
-    <col width="35" customWidth="1" min="19" max="19"/>
-    <col width="35" customWidth="1" min="20" max="20"/>
-    <col width="35" customWidth="1" min="21" max="21"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="36" customWidth="1" min="17" max="17"/>
+    <col width="36" customWidth="1" min="18" max="18"/>
+    <col width="36" customWidth="1" min="19" max="19"/>
+    <col width="36" customWidth="1" min="20" max="20"/>
+    <col width="36" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -579,7 +579,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Code: IAP491_FA26_PI_GUARD | Supervisor: MSc. Supervisor / FPT University IA Department</t>
+          <t>Code: IAP491_FA26_PI_GUARD | Học kỳ Fall 2026 (07/09/2026 – 20/12/2026) | Khoa An toàn Thông tin - Đại học FPT</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       <c r="F4" s="4" t="n"/>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Tiến độ thực hiện hàng tuần (Tuần 1 - Tuần 15)</t>
+          <t>Tiến độ thực hiện hàng tuần (Tuần 1: 07/09/2026 – Tuần 15: 20/12/2026)</t>
         </is>
       </c>
       <c r="H4" s="4" t="n"/>
@@ -629,7 +629,7 @@
       <c r="T4" s="4" t="n"/>
       <c r="U4" s="4" t="n"/>
     </row>
-    <row r="5" ht="25" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="n"/>
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="5" t="inlineStr">
@@ -654,81 +654,96 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 1</t>
+          <t>Tuần 1
+(07/09 - 13/09)</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 2</t>
+          <t>Tuần 2
+(14/09 - 20/09)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 3</t>
+          <t>Tuần 3
+(21/09 - 27/09)</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 4</t>
+          <t>Tuần 4
+(28/09 - 04/10)</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 5</t>
+          <t>Tuần 5
+(05/10 - 11/10)</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 6</t>
+          <t>Tuần 6
+(12/10 - 18/10)</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 7</t>
+          <t>Tuần 7
+(19/10 - 25/10)</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 8</t>
+          <t>Tuần 8
+(26/10 - 01/11)</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 9</t>
+          <t>Tuần 9
+(02/11 - 08/11)</t>
         </is>
       </c>
       <c r="P5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 10</t>
+          <t>Tuần 10
+(09/11 - 15/11)</t>
         </is>
       </c>
       <c r="Q5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 11</t>
+          <t>Tuần 11
+(16/11 - 22/11)</t>
         </is>
       </c>
       <c r="R5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 12</t>
+          <t>Tuần 12
+(23/11 - 29/11)</t>
         </is>
       </c>
       <c r="S5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 13</t>
+          <t>Tuần 13
+(30/11 - 06/12)</t>
         </is>
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 14</t>
+          <t>Tuần 14
+(07/12 - 13/12)</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>Tuần 15</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="90" customHeight="1">
+          <t>Tuần 15
+(14/12 - 20/12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="110" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>SE182034</t>
@@ -761,92 +776,126 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Khởi động đồ án:
-- Đăng ký đề tài PI-Guard với GVHD.
-- Phân công nhiệm vụ 4 thành viên.
-- Thiết lập cấu trúc repo Git.</t>
+          <t>Khởi động &amp; Sàng lọc Papers:
+- Họp GVHD Meeting 1 (29/08) &amp; Meeting 2 (01/09).
+- Đọc &amp; sàng lọc 10 papers theo Register.
+- Cập nhật cơ sở lý thuyết Chapter 1&amp;2.</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Khảo sát &amp; Bối cảnh:
-- Khảo sát OWASP LLM01:2025 &amp; NIST AI 100-2e2025.
-- Thu thập 17 papers tham khảo &gt;= 2022.
-- Soạn thảo Background &amp; Problem Statement.</t>
+          <t>Bối cảnh &amp; Phân loại:
+- Soạn thảo Chapter 1 (Introduction).
+- Phân loại Threat Taxonomy (OWASP).
+- Lỗ hổng Von Neumann NLP.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Hoàn thành Review 1:
-- Hoàn thiện Report No.1 (Introduction).
-- Phân tích Threat Taxonomy.
-- Chuẩn bị slide PPT Review 1 và bảo vệ trước GVHD.</t>
+          <t>Literature Review:
+- Soạn thảo Chapter 2 (Literature Review).
+- Khảo sát SOTA Guardrails.
+- Dàn ý slide 9 trang Review 1.</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Báo cáo No.2 (Literature Review):
-- Khảo sát SOTA Guardrails (ProtectAI, Llama Guard, NeMo).
-- Viết Report No.2 nộp GVHD.</t>
+          <t>BẢO VỆ REVIEW 1 (GVHD):
+- Hoàn thiện Report No.1 &amp; No.2.
+- Thiết kế Slide PPTX &amp; tập diễn tập.
+- Bảo vệ thành công Review 1.</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Data Engineering:
+- Tải 5 datasets từ Hugging Face.
+- Cài đặt Group-Aware Split.
+- Làm sạch &amp; khử trùng lặp dữ liệu.</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Hỗ trợ Baseline ML:
+- Phân tích phân phối nhãn dữ liệu.
+- Đo lường độ rò rỉ Inter-cluster.
+- Hỗ trợ xây dựng baseline TF-IDF.</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Soạn thảo &amp; Cập nhật Docs:
+- Soạn thảo Chapter 3 (Methodology).
+- Tổng hợp cấu trúc Report No.3.
+- Chuẩn bị tài liệu &amp; slide Review 2.</t>
         </is>
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>BẢO VỆ REVIEW 2 (GVHD):
+- Báo cáo Chapter 3 (Methodology &amp; ML).
+- Tiếp thu góp ý &amp; cập nhật hoàn thiện docs.
+- Nghiệm thu Report No.3 (20% điểm).</t>
         </is>
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Transformer Training:
+- Hỗ trợ fine-tuning DeBERTa-v3.
+- Phân tích Attention Weight.
+- Đánh giá độ bền Adversarial.</t>
         </is>
       </c>
       <c r="P6" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Hoàn thiện Report No.4:
+- Đo lường chỉ số F1, FPR trên CPU.
+- Kiểm toán kết quả nén ONNX INT8.
+- Nộp Report No.4 cho GVHD.</t>
         </is>
       </c>
       <c r="Q6" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Tích hợp API Middleware:
+- Điều phối tích hợp FastAPI proxy.
+- Đo latency end-to-end P95 &lt; 30ms.
+- Dựng dashboard Streamlit.</t>
         </is>
       </c>
       <c r="R6" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Chuẩn bị Hội Đồng 1:
+- Hoàn thiện tài liệu kỹ thuật demo.
+- Tổng duyệt Prototype &amp; Slide Hội đồng.
+- Kiểm tra độ ổn định hệ thống.</t>
         </is>
       </c>
       <c r="S6" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>BÁO CÁO HỘI ĐỒNG 1 (MIDTERM):
+- Bảo vệ Prototype Demo trước Hội đồng.
+- Báo cáo kết quả thực nghiệm Chapter 4.
+- Tiếp thu ý kiến phản biện Hội đồng.</t>
         </is>
       </c>
       <c r="T6" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Discussion, Conclusion &amp; Thesis:
+- Soạn thảo Report No.5 &amp; No.6.
+- Tổng hợp Master Thesis 6 chương.
+- Quét Turnitin (&lt; 20%), duyệt Slide.</t>
         </is>
       </c>
       <c r="U6" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="90" customHeight="1">
+          <t>BÁO CÁO HỘI ĐỒNG FINAL (TỐT NGHIỆP):
+- Tổng duyệt Slide PPTX bảo vệ.
+- BẢO VỆ CHÍNH THỨC TRƯỚC HỘI ĐỒNG.
+- Hoàn tất hồ sơ tốt nghiệp FPT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="110" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>SE182087</t>
@@ -879,89 +928,126 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Thiết lập môi trường ML:
-- Cài đặt Python 3.11, Scikit-learn, PyTorch.
-- Tìm hiểu cơ chế Word/Char TF-IDF.</t>
+          <t>Khảo sát ML &amp; JailGuard:
+- Tham gia Meeting 1 &amp; Meeting 2 (01/09).
+- Đọc &amp; phân tích JailGuard (TOSEM 2025).
+- Tìm hiểu Targeted Mutators Workflow.</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Threat Model &amp; Robustness:
-- Xây dựng sơ đồ Threat Model &amp; Attack Surface.
-- Phân tích cơ chế kháng nhiễu Leetspeak/Base64.</t>
+          <t>Threat Model &amp; Attack Surface:
+- Xây dựng sơ đồ NIST AI 100-2e2025.
+- Khóa chặt Attack Surface /v1/chat.
+- Thiết kế kiến trúc bảo vệ 3 lớp.</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Hoàn thành Review 1:
-- Chuẩn bị slide Threat Model &amp; Kiến trúc 3 lớp.
-- Bắt đầu xây dựng baseline TF-IDF script.</t>
+          <t>Chuẩn bị Review 1:
+- Chuẩn bị slide Threat Model &amp; 3L.
+- Xây dựng script baseline TF-IDF mẫu.
+- Thử nghiệm feature extraction.</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Baseline Training:
-- Huấn luyện mô hình Logistic Regression, LinearSVC trên tập train.
-- Đánh giá F1 ban đầu.</t>
+          <t>BẢO VỆ REVIEW 1 (GVHD):
+- Trình bày Threat Model &amp; Kiến trúc 3L.
+- Phản biện phương pháp luận baseline.
+- Hoàn thành mốc Review 1.</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Trích xuất đặc trưng:
+- Xây dựng Word+Char TF-IDF pipeline.
+- Tối ưu hóa sublinear_tf, max_features.
+- Xử lý bộ tiền lọc Base64/Leet.</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Huấn luyện Baseline ML:
+- Huấn luyện LR, LinearSVC, XGBoost.
+- Đánh giá F1, FPR, độ trễ CPU.
+- So sánh hiệu năng các mô hình.</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Methodology &amp; Baseline ML:
+- Soạn thảo chi tiết Chapter 3.
+- Tổng hợp số liệu F1/FPR Baseline.
+- Cập nhật tài liệu kỹ thuật TF-IDF.</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>BẢO VỆ REVIEW 2 (GVHD):
+- Thuyết trình phương pháp luận Chapter 3.
+- Demo kết quả Baseline ML (LR, SVC, XGB).
+- Cập nhật docs theo góp ý của Thầy.</t>
         </is>
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Phân tích Robustness:
+- Đánh giá khả năng chống nhiễu ký tự.
+- Kiểm thử bộ lọc Base64 decoder.
+- Hỗ trợ đánh giá DeBERTa-v3.</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Báo cáo No.4:
+- Tổng hợp số liệu đối chuẩn Baseline.
+- Vẽ biểu đồ ROC-AUC, Confusion Matrix.
+- Đóng góp phần Methodology Report 4.</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Tích hợp Model vào API:
+- Đóng gói mô hình joblib sang API.
+- Viết routing xử lý phân loại nhanh.
+- Kiểm thử latency tầng baseline.</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Chuẩn bị Hội Đồng 1:
+- Đóng gói tài liệu trích xuất đặc trưng.
+- Kiểm thử chéo mô hình Baseline vs ONNX.
+- Tham gia tổng duyệt demo.</t>
         </is>
       </c>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>BÁO CÁO HỘI ĐỒNG 1 (MIDTERM):
+- Trình bày kiến trúc ML &amp; kết quả.
+- Phản biện thuật toán trích xuất đặc trưng.
+- Tiếp thu ý kiến Hội đồng.</t>
         </is>
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Soạn thảo Luận văn:
+- Soạn thảo chuyên sâu Chapter 3 &amp; 4.
+- So sánh ưu nhược TF-IDF vs Transformer.
+- Viết phần thảo luận giới hạn mô hình.</t>
         </is>
       </c>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="90" customHeight="1">
+          <t>BÁO CÁO HỘI ĐỒNG FINAL (TỐT NGHIỆP):
+- Phụ trách báo cáo phần Methodology.
+- Trả lời chất vấn của Hội đồng.
+- Bảo vệ tốt nghiệp xuất sắc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="110" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>SE181851</t>
@@ -994,89 +1080,126 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Khảo sát Transformer:
-- Tìm hiểu DeBERTa-v3 architecture.
-- Khảo sát mô hình tham chiếu ProtectAI DeBERTa.</t>
+          <t>Khảo sát RAP-ID &amp; BIPIA:
+- Tham gia Meeting 1 &amp; Meeting 2 (01/09).
+- Phân tích Pre-fill pass (RAP-ID) &amp; BIPIA.
+- Tìm cơ sở khoa học DeBERTa &lt; 600M.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Ma trận chọn mô hình:
+          <t>SOTA Matrix &amp; Target LLM:
 - Xây dựng Model Selection Matrix.
-- Thiết lập benchmark 5 Target LLM qua Cloud API (GPT-4o, Gemini, LLaMA-3.1).</t>
+- Thiết lập benchmark 5 Target LLMs.
+- Soạn thảo phân tích đối chuẩn.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Hoàn thành Review 1:
-- Xây dựng ma trận 4 Demo kịch bản (2x2).
-- Thử nghiệm đo độ trễ Latency trên CPU.</t>
+          <t>Demo Scenarios Review 1:
+- Thiết kế ma trận 4 Kịch bản Demo 2x2.
+- Viết kịch bản tấn công Prompt Injection.
+- Chuẩn bị slide trình bày SOTA.</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Fine-tuning Transformer:
-- Chuẩn bị pipeline huấn luyện DeBERTa-v3 trên GPU Colab/Kaggle.
-- Chạy baseline test.</t>
+          <t>BẢO VỆ REVIEW 1 (GVHD):
+- Trình bày Model Selection &amp; Demo 2x2.
+- Bảo vệ lựa chọn DeBERTa-v3.
+- Hoàn thành mốc Review 1.</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Chuẩn bị Fine-Tuning:
+- Chuẩn bị dataloader cho Transformer.
+- Thiết lập pipeline tokenize độ dài 512.
+- Cấu hình hyperparameters AdamW/Cosine.</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Khảo sát Baseline &amp; Transformer:
+- Hỗ trợ đánh giá Baseline ML.
+- Khảo sát Disentangled Attention.
+- Chuẩn bị cấu trúc Chapter 3.</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Hỗ trợ Thực nghiệm &amp; Docs:
+- Soạn thảo cấu trúc Chapter 3.
+- Chuẩn bị ma trận đánh giá đối chuẩn.
+- Kiểm tra tính nhất quán dữ liệu.</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>BẢO VỆ REVIEW 2 &amp; Khởi động SFT:
+- Báo cáo định hướng DeBERTa-v3.
+- Cập nhật docs Chapter 3 sau Review 2.
+- Thiết lập pipeline fine-tuning GPU.</t>
         </is>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Fine-Tuning DeBERTa-v3:
+- Huấn luyện DeBERTa-v3 trên GPU.
+- Tối ưu BCEWithLogitsLoss chống lệch nhãn.
+- Theo dõi validation loss &amp; F1-score.</t>
         </is>
       </c>
       <c r="P8" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Lượng hóa ONNX INT8:
+- Xuất mô hình sang ONNX Runtime.
+- Áp dụng dynamic INT8 quantization.
+- Đạt độ trễ P95 &lt; 30ms trên CPU. Nộp R4.</t>
         </is>
       </c>
       <c r="Q8" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Tích hợp Engine ONNX:
+- Viết wrapper suy luận ONNX cho API.
+- Tối ưu hóa đa luồng CPU (OMP_NUM_THREADS).
+- Đo đạc thông lượng xử lý RPS.</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Chuẩn bị Hội Đồng 1:
+- Kiểm thử hiệu năng ONNX trên máy trạm.
+- Chuẩn bị slide thực nghiệm Chapter 4.
+- Tổng duyệt phần trình bày AI Model.</t>
         </is>
       </c>
       <c r="S8" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>BÁO CÁO HỘI ĐỒNG 1 (MIDTERM):
+- Trình diễn trực tiếp mô hình ONNX INT8.
+- Chứng minh độ trễ P95 &lt; 30ms trên CPU.
+- Bảo vệ thành công Prototype.</t>
         </is>
       </c>
       <c r="T8" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Biên soạn Kết quả Thực nghiệm:
+- Viết chi tiết toàn văn Chapter 4.
+- Bảng đối chuẩn F1, FPR, Latency.
+- Phân tích trade-off độ chính xác - tốc độ.</t>
         </is>
       </c>
       <c r="U8" s="6" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="90" customHeight="1">
+          <t>BÁO CÁO HỘI ĐỒNG FINAL (TỐT NGHIỆP):
+- Trình bày kiến trúc DeBERTa &amp; ONNX INT8.
+- Trả lời chất vấn chuyên sâu về AI Security.
+- Hoàn thành xuất sắc đồ án.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="110" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>SE180235</t>
@@ -1109,85 +1232,122 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Khảo sát hạ tầng API:
-- Thiết lập khung dự án FastAPI &amp; Streamlit.
-- Thiết kế kiến trúc proxy chuyển tiếp LLM.</t>
+          <t>Khảo sát Jailbreak &amp; Do-Not-Answer:
+- Tham gia Meeting 1 &amp; Meeting 2 (01/09).
+- Phân loại 3 chiến thuật Jailbreak (Survey).
+- Khảo sát Do-Not-Answer &amp; Black-box def.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Research Questions &amp; Scope:
-- Soạn thảo 3 Câu hỏi nghiên cứu cốt lõi chuẩn IEEE.
-- Phân định rõ ràng ranh giới In-scope / Out-of-scope.</t>
+          <t>Research Questions &amp; Gaps:
+- Soạn thảo 3 Câu hỏi IEEE (RQ1-RQ3).
+- Xác định 3 Gaps &amp; 4 Đóng góp mới.
+- Định vị ranh giới In-scope/Out-of-scope.</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>Hoàn thành Review 1:
-- Thiết kế bộ slide 9 trang Review1_Presentation_Slides_Outline.md.
-- Dựng demo UI mô phỏng 4 kịch bản.</t>
+          <t>Slide Outline Review 1:
+- Thiết kế bộ slide 9 trang Review 1.
+- Dựng demo UI mô phỏng 4 kịch bản.
+- Soạn kịch bản thuyết trình 15 phút.</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Phát triển API Middleware:
-- Hoàn thiện endpoint POST /v1/chat/guardrail.
-- Tích hợp mô hình baseline vào API.</t>
+          <t>BẢO VỆ REVIEW 1 (GVHD):
+- Trình bày RQ1-RQ3 &amp; Đóng góp mới.
+- Điều phối trình chiếu slide Review 1.
+- Hoàn thành mốc Review 1.</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Xây dựng API Core:
+- Viết endpoint POST /v1/chat/completions.
+- Xây dựng tầng tiền xử lý regex &amp; decoding.
+- Tích hợp cấu trúc phản hồi chuẩn RFC.</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Tích hợp Baseline vào API:
+- Kết nối mô hình TF-IDF vào middleware.
+- Ghi log request/response vào JSONL.
+- Xử lý bất đồng bộ async/await.</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Kiến trúc Middleware &amp; Docs:
+- Soạn thảo kiến trúc API Chapter 3.
+- Thiết kế bộ slide báo cáo Review 2.
+- Hoàn thiện bản thảo Report No.3.</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>BẢO VỆ REVIEW 2 (GVHD):
+- Trình diễn kết nối API với Baseline ML.
+- Cập nhật docs theo kết luận họp.
+- Bắt đầu dựng Streamlit Dashboard.</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Phát triển Streamlit Dashboard:
+- Dựng UI nhập prompt kiểm thử trực tiếp.
+- Hiển thị nhãn, confidence score, latency.
+- Tạo trang so sánh 4 kịch bản demo.</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Tích hợp ONNX Engine:
+- Kết nối mô hình ONNX INT8 vào API.
+- Thêm tính năng toggle chuyển đổi mô hình.
+- Tối ưu hóa xử lý lỗi HTTP 400/500.</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Hoàn thiện Dashboard:
+- Thêm biểu đồ phân tích và giám sát log.
+- Dựng dashboard đo latency &amp; throughput.
+- Đóng gói Docker Compose tiện lợi.</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Chuẩn bị Hội Đồng 1:
+- Hoàn thiện UI Dashboard tương tác cao.
+- Viết kịch bản live demo 4 kịch bản.
+- Tổng duyệt kỹ thuật cùng nhóm.</t>
         </is>
       </c>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>BÁO CÁO HỘI ĐỒNG 1 (MIDTERM):
+- Trình chiếu trực tiếp Dashboard &amp; API.
+- Demo tương tác trực quan 4 kịch bản.
+- Tiếp thu góp ý từ Hội đồng Giữa kỳ.</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>Soạn thảo Report No.5 &amp; No.6:
+- Viết Chapter 5 (Discussion &amp; Limitations).
+- Viết Chapter 6 (Conclusion &amp; Future Work).
+- Định dạng chuẩn IEEE/FPT cho Luận văn.</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>[ ] Kế hoạch theo lộ trình</t>
+          <t>BÁO CÁO HỘI ĐỒNG FINAL (TỐT NGHIỆP):
+- Trình bày Demo &amp; Kiến trúc phần mềm.
+- Điều phối phần trình chiếu Hội đồng.
+- Đạt kết quả Tốt nghiệp xuất sắc.</t>
         </is>
       </c>
     </row>
@@ -1211,16 +1371,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -1233,7 +1393,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hướng dẫn: Chọn trạng thái tại cột D từ danh sách thả xuống (Dropdown List)</t>
+          <t>Học kỳ Fall 2026 (07/09/2026 – 20/12/2026) | Hướng dẫn: Chọn trạng thái tại cột D từ danh sách thả xuống</t>
         </is>
       </c>
     </row>
@@ -1282,12 +1442,12 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Tuần 1 (23/08 - 29/08)</t>
+          <t>Tuần 1 (07/09 - 13/09)</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Họp với Giáo viên hướng dẫn (GVHD) và xác định mục tiêu ban đầu (Meeting 1)</t>
+          <t>Họp GVHD định hướng bài toán (Meeting 1_29_08) &amp; Sàng lọc 10 papers khoa học (Meeting 2_01_09)</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
@@ -1297,17 +1457,17 @@
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Trường (Leader)</t>
+          <t>Cả 4 thành viên</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>Biên bản Meeting 1_29_08_26.md</t>
+          <t>Biên bản Meeting 1 &amp; Meeting 2.md</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>29/08/2026</t>
+          <t>13/09/2026</t>
         </is>
       </c>
     </row>
@@ -1319,22 +1479,22 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Tuần 1 (23/08 - 29/08)</t>
+          <t>Tuần 1 (07/09 - 13/09)</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Khảo sát tài liệu nghiên cứu và thu thập 17 papers chuẩn IEEE &gt;= 2022</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+          <t>Thu thập &amp; thẩm định 17 papers chuẩn IEEE &gt;= 2022 theo CAPSTONE REGISTER</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Trường</t>
+          <t>Trường (Leader)</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
@@ -1344,7 +1504,7 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>30/08/2026</t>
+          <t>13/09/2026</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1516,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 2 (14/09 - 20/09)</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -1381,7 +1541,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>31/08/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1553,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 2 (14/09 - 20/09)</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
@@ -1418,7 +1578,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>31/08/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1590,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 2 (14/09 - 20/09)</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -1455,7 +1615,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1627,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 2 (14/09 - 20/09)</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -1492,7 +1652,7 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>19/09/2026</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1664,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 2 (14/09 - 20/09)</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -1529,7 +1689,7 @@
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1701,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 3 (21/09 - 27/09)</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -1566,7 +1726,7 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1738,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 3 (21/09 - 27/09)</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -1603,7 +1763,7 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>03/09/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1775,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 3 (21/09 - 27/09)</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -1640,7 +1800,7 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1812,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 3 (21/09 - 27/09)</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
@@ -1677,7 +1837,7 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>27/09/2026</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1849,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 3 (21/09 - 27/09)</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -1714,7 +1874,7 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>27/09/2026</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1886,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 4 (28/09 - 04/10)</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
@@ -1751,7 +1911,7 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1923,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (30/08 - 05/09)</t>
+          <t>Tuần 4 (28/09 - 04/10)</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
@@ -1788,7 +1948,7 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>06/09/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1960,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Tuần 3 - 4 (06/09 - 19/09)</t>
+          <t>Tuần 4 (28/09 - 04/10)</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
@@ -1825,7 +1985,7 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>Tuần 3-4</t>
+          <t>04/10/2026</t>
         </is>
       </c>
     </row>
@@ -1837,12 +1997,12 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Tuần 5 - 6 (20/09 - 03/10)</t>
+          <t>Tuần 5 - 6 (05/10 - 18/10)</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Thu thập Dataset, Group-Aware Split &amp; Huấn luyện Baseline ML</t>
+          <t>Thu thập Dataset đa nguồn, Group-Aware Split &amp; Huấn luyện Baseline ML</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
@@ -1862,7 +2022,7 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Tuần 6</t>
+          <t>18/10/2026</t>
         </is>
       </c>
     </row>
@@ -1874,12 +2034,12 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Tuần 7 (04/10 - 10/10)</t>
+          <t>Tuần 7 (19/10 - 25/10)</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>CỘT MỐC 2 — Nộp Report No.3 &amp; BẢO VỆ REVIEW 2 TRƯỚC GVHD (CHAPTER 3)</t>
+          <t>Soạn thảo, cập nhật docs Chapter 3 (Methodology - Report No.3) &amp; Chuẩn bị Slide Review 2</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
@@ -1894,12 +2054,12 @@
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>Report No.3 &amp; Demo Baseline</t>
+          <t>docs/thesis/chapters/03_Methodology.md &amp; Slide Review 2</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>Tuần 7</t>
+          <t>25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1911,12 +2071,12 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Tuần 8 - 9 (11/10 - 24/10)</t>
+          <t>Tuần 8 (26/10 - 01/11)</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Fine-tuning DeBERTa-v3, Lượng hóa ONNX INT8 &amp; Nộp Report No.4</t>
+          <t>CỘT MỐC 2 — BẢO VỆ REVIEW 2 TRƯỚC GVHD (CHAPTER 3), Nộp Report No.3 &amp; Cập nhật Docs hoàn chỉnh</t>
         </is>
       </c>
       <c r="D22" s="13" t="inlineStr">
@@ -1926,17 +2086,17 @@
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>Việt &amp; Đức</t>
+          <t>Cả 4 thành viên</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>Report No.4 &amp; models/onnx/</t>
+          <t>Biên bản nghiệm thu Review 2 &amp; Chapter 3 final</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Tuần 9</t>
+          <t>01/11/2026</t>
         </is>
       </c>
     </row>
@@ -1948,12 +2108,12 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Tuần 10 - 12 (25/10 - 14/11)</t>
+          <t>Tuần 9 - 10 (02/11 - 15/11)</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>CỘT MỐC 3 — BÁO CÁO HỘI ĐỒNG 1 (HỘI ĐỒNG GIỮA KỲ — PROTOTYPE DEMO)</t>
+          <t>Fine-tuning DeBERTa-v3, Lượng hóa ONNX INT8, Đánh giá Adversarial &amp; Nộp Report No.4</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
@@ -1963,17 +2123,17 @@
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>Phương &amp; Việt</t>
+          <t>Việt &amp; Đức</t>
         </is>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>Hệ thống Prototype hoàn chỉnh</t>
+          <t>Report No.4 &amp; models/onnx/</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>Tuần 12</t>
+          <t>15/11/2026</t>
         </is>
       </c>
     </row>
@@ -1985,12 +2145,12 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Tuần 13 - 15 (15/11 - 05/12)</t>
+          <t>Tuần 11 - 12 (16/11 - 29/11)</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>CỘT MỐC 4 — BÁO CÁO HỘI ĐỒNG FINAL (BẢO VỆ TỐT NGHIỆP TOÀN DIỆN 6 CHƯƠNG)</t>
+          <t>Xây dựng API Middleware, Streamlit Dashboard &amp; Tích hợp Prototype Demo 3 lớp</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
@@ -2000,17 +2160,128 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
+          <t>Phương &amp; Việt</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Hệ thống Prototype hoàn chỉnh</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>29/11/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="25" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Tuần 13 (30/11 - 06/12)</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>CỘT MỐC 3 — BÁO CÁO HỘI ĐỒNG 1 (HỘI ĐỒNG GIỮA KỲ — PROTOTYPE DEMO &amp; CHAPTER 4)</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
           <t>Cả 4 thành viên</t>
         </is>
       </c>
-      <c r="F24" s="10" t="inlineStr">
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Biên bản nghiệm thu Hội đồng 1</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>06/12/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="25" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Tuần 14 (07/12 - 13/12)</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Soạn Report No.5 &amp; No.6, Tổng hợp Master Thesis 6 chương qua script &amp; Quét Turnitin (&lt; 20%)</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Cả 4 thành viên</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>FINAL_THESIS.md &amp; Report 5, 6</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>13/12/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="25" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Tuần 15 (14/12 - 20/12)</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>CỘT MỐC 4 — BẢO VỆ TỐT NGHIỆP TOÀN DIỆN 6 CHƯƠNG TRƯỚC HỘI ĐỒNG FINAL</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Cả 4 thành viên</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
         <is>
           <t>Final Thesis &amp; Slide Defense</t>
         </is>
       </c>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>Tuần 15</t>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>20/12/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(workspaces): simplify member folders to truongnv, ducnq, vietpmh, phuongddd and fix CI badge in README
</commit_message>
<xml_diff>
--- a/Meeting/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/Meeting/PI_GUARD_PROCESS_REPORT.xlsx
@@ -1536,7 +1536,7 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>workspaces/truong_data_eng/docs/</t>
+          <t>workspaces/truongnv/docs/</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>workspaces/truong_data_eng/docs/</t>
+          <t>workspaces/truongnv/docs/</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>workspaces/duc_baseline_ml/</t>
+          <t>workspaces/ducnq/</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>workspaces/duc_baseline_ml/</t>
+          <t>workspaces/ducnq/</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>workspaces/phuong_api_dashboard/</t>
+          <t>workspaces/phuongddd/</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>workspaces/viet_transformer_robustness/</t>
+          <t>workspaces/vietpmh/</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>workspaces/viet_transformer_robustness/</t>
+          <t>workspaces/vietpmh/</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>workspaces/truong_data_eng/docs/</t>
+          <t>workspaces/truongnv/docs/</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>workspaces/truong_data_eng/docs/</t>
+          <t>workspaces/truongnv/docs/</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>workspaces/truong_data_eng/docs/</t>
+          <t>workspaces/truongnv/docs/</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">

</xml_diff>

<commit_message>
refactor(review1): ground review 1 scope to literature review and illustrative scenarios without premature empirical claims
</commit_message>
<xml_diff>
--- a/Meeting/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/Meeting/PI_GUARD_PROCESS_REPORT.xlsx
@@ -1088,25 +1088,25 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>SOTA Matrix &amp; Target LLM:
-- Xây dựng Model Selection Matrix.
-- Thiết lập benchmark 5 Target LLMs.
-- Soạn thảo phân tích đối chuẩn.</t>
+          <t>Khảo sát Y văn Guardrail:
+- Đối sánh các trường phái Guardrail.
+- Khảo sát các dòng Target LLMs.
+- Soạn thảo luận giải chọn mô hình.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Demo Scenarios Review 1:
+          <t>Kịch bản Minh họa Đề bài:
 - Thiết kế ma trận 4 Kịch bản Demo 2x2.
-- Viết kịch bản tấn công Prompt Injection.
-- Chuẩn bị slide trình bày SOTA.</t>
+- Xây dựng luồng tấn công vs đề xuất bảo vệ.
+- Chuẩn bị slide thuyết trình Review 1.</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
           <t>BẢO VỆ REVIEW 1 (GVHD):
-- Trình bày Model Selection &amp; Demo 2x2.
-- Bảo vệ lựa chọn DeBERTa-v3.
+- Trình bày Luận giải mô hình &amp; Demo đề bài.
+- Báo cáo cơ sở khoa học DeBERTa-v3.
 - Hoàn thành mốc Review 1.</t>
         </is>
       </c>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Khảo sát SOTA Guardrails, Model Selection Matrix &amp; Benchmark 5 Target LLMs</t>
+          <t>Khảo sát SOTA Guardrails, Luận giải chọn mô hình &amp; Khảo sát 5 Target LLMs</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Thiết kế &amp; kiểm thử Ma trận 4 Kịch bản Demo (2x2: Vulnerable vs Protected)</t>
+          <t>Thiết kế Ma trận 4 Kịch bản Minh họa Đề bài (2x2: Vulnerable vs Proposed Protected)</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">

</xml_diff>